<commit_message>
Restructure READMEs + fix event windows + update results
- Rewrote README.md and README_EN.md with new structure: research questions
  first, then core findings (H1/H2 with actual numbers and embedded figures),
  then background, data, methodology, results, robustness, discussion, limitations
- Fixed event study methodology: removed windows overlapping estimation window
  [-5,+60] and [-20,+60]; replaced with clean windows [-1,+1], [0,+5],
  [0,+10], [0,+20], [0,+60] starting at t=-1 or later
- Added CAAR time path plot (fig_caar_path_full.png, t=-11 to +60)
- Updated DID tables to use new window names; added [0,+60] as long-run window
- Regenerated car_summary.csv, car_by_event.csv, FINAL_RESULTS.xlsx
- Added Core Tech subsample (N=182) as second named subsample in data section

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/results/FINAL_RESULTS.xlsx
+++ b/data/results/FINAL_RESULTS.xlsx
@@ -446,12 +446,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L57"/>
+  <dimension ref="A1:L46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
     <col width="8" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
     <col width="6" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="11" customWidth="1" min="6" max="6"/>
@@ -571,7 +571,7 @@
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>-3.297</t>
+          <t>-3.298</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
@@ -598,7 +598,7 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>[-20,+60]</t>
+          <t>[0,+10]</t>
         </is>
       </c>
       <c r="D3" s="2" t="n">
@@ -606,42 +606,42 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>4.668***</t>
+          <t>0.093**</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>3.064</t>
+          <t>-1.365</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>0.0022</t>
+          <t>0.1723</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>2.240</t>
+          <t>-0.894</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>0.0256</t>
+          <t>0.3719</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>0.356</t>
+          <t>-2.187</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>0.7221</t>
+          <t>0.0287</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>***</t>
+          <t>**</t>
         </is>
       </c>
     </row>
@@ -658,7 +658,7 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>[-5,+60]</t>
+          <t>[0,+20]</t>
         </is>
       </c>
       <c r="D4" s="2" t="n">
@@ -666,44 +666,40 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>5.097***</t>
+          <t>1.300</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>3.626</t>
+          <t>1.107</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>0.0003</t>
+          <t>0.2681</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>2.558</t>
+          <t>0.789</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>0.0109</t>
+          <t>0.4306</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>0.313</t>
+          <t>-0.828</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
         <is>
-          <t>0.7546</t>
-        </is>
-      </c>
-      <c r="L4" s="2" t="inlineStr">
-        <is>
-          <t>***</t>
-        </is>
-      </c>
+          <t>0.4078</t>
+        </is>
+      </c>
+      <c r="L4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -718,7 +714,7 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>[0,+10]</t>
+          <t>[0,+5]</t>
         </is>
       </c>
       <c r="D5" s="2" t="n">
@@ -726,42 +722,42 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>0.093**</t>
+          <t>-0.658***</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>-1.365</t>
+          <t>-3.267</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>0.1723</t>
+          <t>0.0011</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>-0.894</t>
+          <t>-1.966</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>0.3719</t>
+          <t>0.0499</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>-2.213</t>
+          <t>-2.711</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
         <is>
-          <t>0.0269</t>
+          <t>0.0067</t>
         </is>
       </c>
       <c r="L5" s="2" t="inlineStr">
         <is>
-          <t>**</t>
+          <t>***</t>
         </is>
       </c>
     </row>
@@ -778,7 +774,7 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>[0,+1]</t>
+          <t>[0,+60]</t>
         </is>
       </c>
       <c r="D6" s="2" t="n">
@@ -786,12 +782,12 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>-0.700***</t>
+          <t>5.335***</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>-4.986</t>
+          <t>4.093</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -801,22 +797,22 @@
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>-2.128</t>
+          <t>2.861</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>0.0339</t>
+          <t>0.0044</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>-2.736</t>
+          <t>0.775</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
         <is>
-          <t>0.0062</t>
+          <t>0.4386</t>
         </is>
       </c>
       <c r="L6" s="2" t="inlineStr">
@@ -828,7 +824,7 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>US only (PRIMARY)</t>
+          <t>Core tech, US only</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
@@ -838,53 +834,57 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>[0,+20]</t>
+          <t>[-1,+1]</t>
         </is>
       </c>
       <c r="D7" s="2" t="n">
-        <v>429</v>
+        <v>182</v>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>1.300</t>
+          <t>-1.015***</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>1.107</t>
+          <t>-3.636</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>0.2681</t>
+          <t>0.0003</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>0.789</t>
+          <t>-1.829</t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>0.4306</t>
+          <t>0.0690</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>-0.863</t>
+          <t>-1.731</t>
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr">
         <is>
-          <t>0.3883</t>
-        </is>
-      </c>
-      <c r="L7" s="2" t="inlineStr"/>
+          <t>0.0835</t>
+        </is>
+      </c>
+      <c r="L7" s="2" t="inlineStr">
+        <is>
+          <t>***</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>US only (PRIMARY)</t>
+          <t>Core tech, US only</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
@@ -894,50 +894,50 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>[0,+5]</t>
+          <t>[0,+10]</t>
         </is>
       </c>
       <c r="D8" s="2" t="n">
-        <v>429</v>
+        <v>182</v>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>-0.658***</t>
+          <t>-0.261*</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>-3.267</t>
+          <t>-1.395</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>0.0011</t>
+          <t>0.1630</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>-1.966</t>
+          <t>-0.803</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>0.0499</t>
+          <t>0.4227</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>-2.730</t>
+          <t>-1.682</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr">
         <is>
-          <t>0.0063</t>
+          <t>0.0925</t>
         </is>
       </c>
       <c r="L8" s="2" t="inlineStr">
         <is>
-          <t>***</t>
+          <t>*</t>
         </is>
       </c>
     </row>
@@ -954,7 +954,7 @@
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>[-1,+1]</t>
+          <t>[0,+20]</t>
         </is>
       </c>
       <c r="D9" s="2" t="n">
@@ -962,42 +962,42 @@
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>-1.015***</t>
+          <t>2.222**</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>-3.636</t>
+          <t>2.028</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>0.0003</t>
+          <t>0.0426</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>-1.829</t>
+          <t>1.264</t>
         </is>
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>0.0690</t>
+          <t>0.2077</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>-1.739</t>
+          <t>-0.196</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr">
         <is>
-          <t>0.0821</t>
+          <t>0.8448</t>
         </is>
       </c>
       <c r="L9" s="2" t="inlineStr">
         <is>
-          <t>***</t>
+          <t>**</t>
         </is>
       </c>
     </row>
@@ -1014,7 +1014,7 @@
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>[-20,+60]</t>
+          <t>[0,+5]</t>
         </is>
       </c>
       <c r="D10" s="2" t="n">
@@ -1022,37 +1022,37 @@
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>4.696**</t>
+          <t>-0.516**</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>2.408</t>
+          <t>-2.180</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>0.0160</t>
+          <t>0.0292</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>1.465</t>
+          <t>-1.270</t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>0.1446</t>
+          <t>0.2059</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>0.401</t>
+          <t>-1.617</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr">
         <is>
-          <t>0.6888</t>
+          <t>0.1060</t>
         </is>
       </c>
       <c r="L10" s="2" t="inlineStr">
@@ -1074,7 +1074,7 @@
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>[-5,+60]</t>
+          <t>[0,+60]</t>
         </is>
       </c>
       <c r="D11" s="2" t="n">
@@ -1082,37 +1082,37 @@
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>5.308***</t>
+          <t>5.854***</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>2.916</t>
+          <t>3.463</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>0.0035</t>
+          <t>0.0005</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>1.731</t>
+          <t>2.036</t>
         </is>
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>0.0851</t>
+          <t>0.0432</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>0.270</t>
+          <t>0.652</t>
         </is>
       </c>
       <c r="K11" s="2" t="inlineStr">
         <is>
-          <t>0.7874</t>
+          <t>0.5145</t>
         </is>
       </c>
       <c r="L11" s="2" t="inlineStr">
@@ -1124,7 +1124,7 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Core tech, US only</t>
+          <t>Non-tech, US only</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
@@ -1134,57 +1134,57 @@
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>[0,+10]</t>
+          <t>[-1,+1]</t>
         </is>
       </c>
       <c r="D12" s="2" t="n">
-        <v>182</v>
+        <v>247</v>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>-0.261*</t>
+          <t>-0.921***</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>-1.395</t>
+          <t>-3.837</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>0.1630</t>
+          <t>0.0001</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>-0.803</t>
+          <t>-1.765</t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>0.4227</t>
+          <t>0.0789</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>-1.710</t>
+          <t>-2.833</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr">
         <is>
-          <t>0.0872</t>
+          <t>0.0046</t>
         </is>
       </c>
       <c r="L12" s="2" t="inlineStr">
         <is>
-          <t>*</t>
+          <t>***</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Core tech, US only</t>
+          <t>Non-tech, US only</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
@@ -1194,57 +1194,53 @@
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>[0,+1]</t>
+          <t>[0,+10]</t>
         </is>
       </c>
       <c r="D13" s="2" t="n">
-        <v>182</v>
+        <v>247</v>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>-0.761***</t>
+          <t>0.354</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>-3.622</t>
+          <t>-0.601</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>0.0003</t>
+          <t>0.5478</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>-1.549</t>
+          <t>-0.444</t>
         </is>
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>0.1232</t>
+          <t>0.6577</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>-1.637</t>
+          <t>-1.424</t>
         </is>
       </c>
       <c r="K13" s="2" t="inlineStr">
         <is>
-          <t>0.1016</t>
-        </is>
-      </c>
-      <c r="L13" s="2" t="inlineStr">
-        <is>
-          <t>***</t>
-        </is>
-      </c>
+          <t>0.1545</t>
+        </is>
+      </c>
+      <c r="L13" s="2" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Core tech, US only</t>
+          <t>Non-tech, US only</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
@@ -1258,53 +1254,49 @@
         </is>
       </c>
       <c r="D14" s="2" t="n">
-        <v>182</v>
+        <v>247</v>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>2.222**</t>
+          <t>0.621</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>2.028</t>
+          <t>-0.281</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>0.0426</t>
+          <t>0.7785</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>1.264</t>
+          <t>-0.228</t>
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>0.2077</t>
+          <t>0.8200</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>-0.238</t>
+          <t>-0.930</t>
         </is>
       </c>
       <c r="K14" s="2" t="inlineStr">
         <is>
-          <t>0.8115</t>
-        </is>
-      </c>
-      <c r="L14" s="2" t="inlineStr">
-        <is>
-          <t>**</t>
-        </is>
-      </c>
+          <t>0.3522</t>
+        </is>
+      </c>
+      <c r="L14" s="2" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Core tech, US only</t>
+          <t>Non-tech, US only</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
@@ -1318,41 +1310,41 @@
         </is>
       </c>
       <c r="D15" s="2" t="n">
-        <v>182</v>
+        <v>247</v>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>-0.516**</t>
+          <t>-0.763**</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>-2.180</t>
+          <t>-2.434</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>0.0292</t>
+          <t>0.0149</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>-1.270</t>
+          <t>-1.500</t>
         </is>
       </c>
       <c r="I15" s="2" t="inlineStr">
         <is>
-          <t>0.2059</t>
+          <t>0.1350</t>
         </is>
       </c>
       <c r="J15" s="2" t="inlineStr">
         <is>
-          <t>-1.636</t>
+          <t>-2.177</t>
         </is>
       </c>
       <c r="K15" s="2" t="inlineStr">
         <is>
-          <t>0.1019</t>
+          <t>0.0295</t>
         </is>
       </c>
       <c r="L15" s="2" t="inlineStr">
@@ -1374,7 +1366,7 @@
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>[-1,+1]</t>
+          <t>[0,+60]</t>
         </is>
       </c>
       <c r="D16" s="2" t="n">
@@ -1382,49 +1374,49 @@
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>-0.921***</t>
+          <t>4.952**</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>-3.837</t>
+          <t>2.421</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>0.0001</t>
+          <t>0.0155</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>-1.765</t>
+          <t>2.027</t>
         </is>
       </c>
       <c r="I16" s="2" t="inlineStr">
         <is>
-          <t>0.0789</t>
+          <t>0.0438</t>
         </is>
       </c>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>-2.825</t>
+          <t>0.448</t>
         </is>
       </c>
       <c r="K16" s="2" t="inlineStr">
         <is>
-          <t>0.0047</t>
+          <t>0.6541</t>
         </is>
       </c>
       <c r="L16" s="2" t="inlineStr">
         <is>
-          <t>***</t>
+          <t>**</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>Non-tech, US only</t>
+          <t>Full sample</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
@@ -1434,57 +1426,57 @@
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>[-20,+60]</t>
+          <t>[-1,+1]</t>
         </is>
       </c>
       <c r="D17" s="2" t="n">
-        <v>247</v>
+        <v>468</v>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>4.647**</t>
+          <t>-0.712***</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>1.971</t>
+          <t>-4.451</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>0.0487</t>
+          <t>0.0000</t>
         </is>
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>1.751</t>
+          <t>-2.165</t>
         </is>
       </c>
       <c r="I17" s="2" t="inlineStr">
         <is>
-          <t>0.0811</t>
+          <t>0.0309</t>
         </is>
       </c>
       <c r="J17" s="2" t="inlineStr">
         <is>
-          <t>0.109</t>
+          <t>-2.561</t>
         </is>
       </c>
       <c r="K17" s="2" t="inlineStr">
         <is>
-          <t>0.9129</t>
+          <t>0.0104</t>
         </is>
       </c>
       <c r="L17" s="2" t="inlineStr">
         <is>
-          <t>**</t>
+          <t>***</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Non-tech, US only</t>
+          <t>Full sample</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
@@ -1494,57 +1486,57 @@
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>[-5,+60]</t>
+          <t>[0,+10]</t>
         </is>
       </c>
       <c r="D18" s="2" t="n">
-        <v>247</v>
+        <v>468</v>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>4.941**</t>
+          <t>0.303*</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>2.275</t>
+          <t>-0.892</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>0.0229</t>
+          <t>0.3727</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>1.919</t>
+          <t>-0.585</t>
         </is>
       </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
-          <t>0.0562</t>
+          <t>0.5592</t>
         </is>
       </c>
       <c r="J18" s="2" t="inlineStr">
         <is>
-          <t>0.173</t>
+          <t>-1.799</t>
         </is>
       </c>
       <c r="K18" s="2" t="inlineStr">
         <is>
-          <t>0.8630</t>
+          <t>0.0721</t>
         </is>
       </c>
       <c r="L18" s="2" t="inlineStr">
         <is>
-          <t>**</t>
+          <t>*</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>Non-tech, US only</t>
+          <t>Full sample</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
@@ -1554,53 +1546,57 @@
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>[0,+10]</t>
+          <t>[0,+20]</t>
         </is>
       </c>
       <c r="D19" s="2" t="n">
-        <v>247</v>
+        <v>468</v>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>0.354</t>
+          <t>1.777*</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>-0.601</t>
+          <t>1.851</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>0.5478</t>
+          <t>0.0641</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>-0.444</t>
+          <t>1.314</t>
         </is>
       </c>
       <c r="I19" s="2" t="inlineStr">
         <is>
-          <t>0.6577</t>
+          <t>0.1895</t>
         </is>
       </c>
       <c r="J19" s="2" t="inlineStr">
         <is>
-          <t>-1.433</t>
+          <t>-0.119</t>
         </is>
       </c>
       <c r="K19" s="2" t="inlineStr">
         <is>
-          <t>0.1519</t>
-        </is>
-      </c>
-      <c r="L19" s="2" t="inlineStr"/>
+          <t>0.9054</t>
+        </is>
+      </c>
+      <c r="L19" s="2" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Non-tech, US only</t>
+          <t>Full sample</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
@@ -1610,45 +1606,45 @@
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>[0,+1]</t>
+          <t>[0,+5]</t>
         </is>
       </c>
       <c r="D20" s="2" t="n">
-        <v>247</v>
+        <v>468</v>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>-0.654***</t>
+          <t>-0.479***</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>-3.461</t>
+          <t>-2.715</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>0.0005</t>
+          <t>0.0066</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>-1.473</t>
+          <t>-1.655</t>
         </is>
       </c>
       <c r="I20" s="2" t="inlineStr">
         <is>
-          <t>0.1421</t>
+          <t>0.0987</t>
         </is>
       </c>
       <c r="J20" s="2" t="inlineStr">
         <is>
-          <t>-2.189</t>
+          <t>-2.246</t>
         </is>
       </c>
       <c r="K20" s="2" t="inlineStr">
         <is>
-          <t>0.0286</t>
+          <t>0.0247</t>
         </is>
       </c>
       <c r="L20" s="2" t="inlineStr">
@@ -1660,7 +1656,7 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>Non-tech, US only</t>
+          <t>Full sample</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
@@ -1670,53 +1666,57 @@
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>[0,+20]</t>
+          <t>[0,+60]</t>
         </is>
       </c>
       <c r="D21" s="2" t="n">
-        <v>247</v>
+        <v>468</v>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>0.621</t>
+          <t>5.749***</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>-0.281</t>
+          <t>4.617</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>0.7785</t>
+          <t>0.0000</t>
         </is>
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t>-0.228</t>
+          <t>3.201</t>
         </is>
       </c>
       <c r="I21" s="2" t="inlineStr">
         <is>
-          <t>0.8200</t>
+          <t>0.0015</t>
         </is>
       </c>
       <c r="J21" s="2" t="inlineStr">
         <is>
-          <t>-0.939</t>
+          <t>1.332</t>
         </is>
       </c>
       <c r="K21" s="2" t="inlineStr">
         <is>
-          <t>0.3478</t>
-        </is>
-      </c>
-      <c r="L21" s="2" t="inlineStr"/>
+          <t>0.1829</t>
+        </is>
+      </c>
+      <c r="L21" s="2" t="inlineStr">
+        <is>
+          <t>***</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>Non-tech, US only</t>
+          <t>US only, Post-GenAI (&gt;=2023)</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
@@ -1726,57 +1726,57 @@
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>[0,+5]</t>
+          <t>[-1,+1]</t>
         </is>
       </c>
       <c r="D22" s="2" t="n">
-        <v>247</v>
+        <v>310</v>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>-0.763**</t>
+          <t>-0.992***</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>-2.434</t>
+          <t>-4.657</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>0.0149</t>
+          <t>0.0000</t>
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>-1.500</t>
+          <t>-2.431</t>
         </is>
       </c>
       <c r="I22" s="2" t="inlineStr">
         <is>
-          <t>0.1350</t>
+          <t>0.0156</t>
         </is>
       </c>
       <c r="J22" s="2" t="inlineStr">
         <is>
-          <t>-2.185</t>
+          <t>-2.886</t>
         </is>
       </c>
       <c r="K22" s="2" t="inlineStr">
         <is>
-          <t>0.0289</t>
+          <t>0.0039</t>
         </is>
       </c>
       <c r="L22" s="2" t="inlineStr">
         <is>
-          <t>**</t>
+          <t>***</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>Full sample</t>
+          <t>US only, Post-GenAI (&gt;=2023)</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
@@ -1786,57 +1786,57 @@
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>[-1,+1]</t>
+          <t>[0,+10]</t>
         </is>
       </c>
       <c r="D23" s="2" t="n">
-        <v>467</v>
+        <v>310</v>
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>-0.706***</t>
+          <t>-0.298**</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>-4.429</t>
+          <t>-2.338</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>0.0000</t>
+          <t>0.0194</t>
         </is>
       </c>
       <c r="H23" s="2" t="inlineStr">
         <is>
-          <t>-2.152</t>
+          <t>-1.622</t>
         </is>
       </c>
       <c r="I23" s="2" t="inlineStr">
         <is>
-          <t>0.0319</t>
+          <t>0.1059</t>
         </is>
       </c>
       <c r="J23" s="2" t="inlineStr">
         <is>
-          <t>-2.555</t>
+          <t>-2.461</t>
         </is>
       </c>
       <c r="K23" s="2" t="inlineStr">
         <is>
-          <t>0.0106</t>
+          <t>0.0139</t>
         </is>
       </c>
       <c r="L23" s="2" t="inlineStr">
         <is>
-          <t>***</t>
+          <t>**</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>Full sample</t>
+          <t>US only, Post-GenAI (&gt;=2023)</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
@@ -1846,57 +1846,53 @@
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>[-20,+60]</t>
+          <t>[0,+20]</t>
         </is>
       </c>
       <c r="D24" s="2" t="n">
-        <v>467</v>
+        <v>310</v>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>5.278***</t>
+          <t>0.873</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>3.582</t>
+          <t>0.083</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>0.0003</t>
+          <t>0.9340</t>
         </is>
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>2.593</t>
+          <t>0.061</t>
         </is>
       </c>
       <c r="I24" s="2" t="inlineStr">
         <is>
-          <t>0.0098</t>
+          <t>0.9516</t>
         </is>
       </c>
       <c r="J24" s="2" t="inlineStr">
         <is>
-          <t>0.898</t>
+          <t>-1.021</t>
         </is>
       </c>
       <c r="K24" s="2" t="inlineStr">
         <is>
-          <t>0.3693</t>
-        </is>
-      </c>
-      <c r="L24" s="2" t="inlineStr">
-        <is>
-          <t>***</t>
-        </is>
-      </c>
+          <t>0.3073</t>
+        </is>
+      </c>
+      <c r="L24" s="2" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>Full sample</t>
+          <t>US only, Post-GenAI (&gt;=2023)</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
@@ -1906,45 +1902,45 @@
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>[-5,+60]</t>
+          <t>[0,+5]</t>
         </is>
       </c>
       <c r="D25" s="2" t="n">
-        <v>467</v>
+        <v>310</v>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>5.639***</t>
+          <t>-0.475***</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>4.161</t>
+          <t>-2.829</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>0.0000</t>
+          <t>0.0047</t>
         </is>
       </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
-          <t>2.911</t>
+          <t>-1.748</t>
         </is>
       </c>
       <c r="I25" s="2" t="inlineStr">
         <is>
-          <t>0.0038</t>
+          <t>0.0814</t>
         </is>
       </c>
       <c r="J25" s="2" t="inlineStr">
         <is>
-          <t>0.831</t>
+          <t>-2.158</t>
         </is>
       </c>
       <c r="K25" s="2" t="inlineStr">
         <is>
-          <t>0.4059</t>
+          <t>0.0309</t>
         </is>
       </c>
       <c r="L25" s="2" t="inlineStr">
@@ -1956,7 +1952,7 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>Full sample</t>
+          <t>US only, Post-GenAI (&gt;=2023)</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
@@ -1966,57 +1962,57 @@
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>[0,+10]</t>
+          <t>[0,+60]</t>
         </is>
       </c>
       <c r="D26" s="2" t="n">
-        <v>467</v>
+        <v>310</v>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>0.296*</t>
+          <t>3.767**</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>-0.906</t>
+          <t>2.082</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>0.3650</t>
+          <t>0.0374</t>
         </is>
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>-0.593</t>
+          <t>1.485</t>
         </is>
       </c>
       <c r="I26" s="2" t="inlineStr">
         <is>
-          <t>0.5532</t>
+          <t>0.1385</t>
         </is>
       </c>
       <c r="J26" s="2" t="inlineStr">
         <is>
-          <t>-1.858</t>
+          <t>0.397</t>
         </is>
       </c>
       <c r="K26" s="2" t="inlineStr">
         <is>
-          <t>0.0631</t>
+          <t>0.6911</t>
         </is>
       </c>
       <c r="L26" s="2" t="inlineStr">
         <is>
-          <t>*</t>
+          <t>**</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>Full sample</t>
+          <t>US only, Pre-GenAI (&lt;=2022)</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
@@ -2026,57 +2022,57 @@
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>[0,+1]</t>
+          <t>[-1,+1]</t>
         </is>
       </c>
       <c r="D27" s="2" t="n">
-        <v>467</v>
+        <v>119</v>
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>-0.551***</t>
+          <t>-0.878**</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>-4.343</t>
+          <t>-2.508</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>0.0000</t>
+          <t>0.0121</t>
         </is>
       </c>
       <c r="H27" s="2" t="inlineStr">
         <is>
-          <t>-1.882</t>
+          <t>-0.999</t>
         </is>
       </c>
       <c r="I27" s="2" t="inlineStr">
         <is>
-          <t>0.0604</t>
+          <t>0.3200</t>
         </is>
       </c>
       <c r="J27" s="2" t="inlineStr">
         <is>
-          <t>-2.245</t>
+          <t>-1.620</t>
         </is>
       </c>
       <c r="K27" s="2" t="inlineStr">
         <is>
-          <t>0.0248</t>
+          <t>0.1053</t>
         </is>
       </c>
       <c r="L27" s="2" t="inlineStr">
         <is>
-          <t>***</t>
+          <t>**</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>Full sample</t>
+          <t>US only, Pre-GenAI (&lt;=2022)</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
@@ -2086,57 +2082,53 @@
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>[0,+20]</t>
+          <t>[0,+10]</t>
         </is>
       </c>
       <c r="D28" s="2" t="n">
-        <v>467</v>
+        <v>119</v>
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>1.761*</t>
+          <t>1.113</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>1.825</t>
+          <t>1.183</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>0.0680</t>
+          <t>0.2369</t>
         </is>
       </c>
       <c r="H28" s="2" t="inlineStr">
         <is>
-          <t>1.294</t>
+          <t>0.686</t>
         </is>
       </c>
       <c r="I28" s="2" t="inlineStr">
         <is>
-          <t>0.1962</t>
+          <t>0.4939</t>
         </is>
       </c>
       <c r="J28" s="2" t="inlineStr">
         <is>
-          <t>-0.197</t>
+          <t>-0.282</t>
         </is>
       </c>
       <c r="K28" s="2" t="inlineStr">
         <is>
-          <t>0.8435</t>
-        </is>
-      </c>
-      <c r="L28" s="2" t="inlineStr">
-        <is>
-          <t>*</t>
-        </is>
-      </c>
+          <t>0.7781</t>
+        </is>
+      </c>
+      <c r="L28" s="2" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>Full sample</t>
+          <t>US only, Pre-GenAI (&lt;=2022)</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
@@ -2146,57 +2138,57 @@
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>[0,+5]</t>
+          <t>[0,+20]</t>
         </is>
       </c>
       <c r="D29" s="2" t="n">
-        <v>467</v>
+        <v>119</v>
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>-0.468***</t>
+          <t>2.414**</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>-2.687</t>
+          <t>1.969</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>0.0072</t>
+          <t>0.0490</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
         <is>
-          <t>-1.636</t>
+          <t>1.311</t>
         </is>
       </c>
       <c r="I29" s="2" t="inlineStr">
         <is>
-          <t>0.1025</t>
+          <t>0.1925</t>
         </is>
       </c>
       <c r="J29" s="2" t="inlineStr">
         <is>
-          <t>-2.239</t>
+          <t>0.031</t>
         </is>
       </c>
       <c r="K29" s="2" t="inlineStr">
         <is>
-          <t>0.0252</t>
+          <t>0.9753</t>
         </is>
       </c>
       <c r="L29" s="2" t="inlineStr">
         <is>
-          <t>***</t>
+          <t>**</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>US only, Post-GenAI (&gt;=2023)</t>
+          <t>US only, Pre-GenAI (&lt;=2022)</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
@@ -2206,57 +2198,57 @@
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>[-1,+1]</t>
+          <t>[0,+5]</t>
         </is>
       </c>
       <c r="D30" s="2" t="n">
-        <v>310</v>
+        <v>119</v>
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>-0.992***</t>
+          <t>-1.136*</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>-4.657</t>
+          <t>-1.636</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>0.0000</t>
+          <t>0.1018</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
         <is>
-          <t>-2.431</t>
+          <t>-0.921</t>
         </is>
       </c>
       <c r="I30" s="2" t="inlineStr">
         <is>
-          <t>0.0156</t>
+          <t>0.3589</t>
         </is>
       </c>
       <c r="J30" s="2" t="inlineStr">
         <is>
-          <t>-2.882</t>
+          <t>-1.664</t>
         </is>
       </c>
       <c r="K30" s="2" t="inlineStr">
         <is>
-          <t>0.0040</t>
+          <t>0.0960</t>
         </is>
       </c>
       <c r="L30" s="2" t="inlineStr">
         <is>
-          <t>***</t>
+          <t>*</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>US only, Post-GenAI (&gt;=2023)</t>
+          <t>US only, Pre-GenAI (&lt;=2022)</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
@@ -2266,57 +2258,57 @@
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>[-20,+60]</t>
+          <t>[0,+60]</t>
         </is>
       </c>
       <c r="D31" s="2" t="n">
-        <v>310</v>
+        <v>119</v>
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>3.497*</t>
+          <t>9.419***</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>1.649</t>
+          <t>4.412</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>0.0991</t>
+          <t>0.0000</t>
         </is>
       </c>
       <c r="H31" s="2" t="inlineStr">
         <is>
-          <t>1.201</t>
+          <t>2.962</t>
         </is>
       </c>
       <c r="I31" s="2" t="inlineStr">
         <is>
-          <t>0.2307</t>
+          <t>0.0037</t>
         </is>
       </c>
       <c r="J31" s="2" t="inlineStr">
         <is>
-          <t>0.079</t>
+          <t>0.807</t>
         </is>
       </c>
       <c r="K31" s="2" t="inlineStr">
         <is>
-          <t>0.9366</t>
+          <t>0.4199</t>
         </is>
       </c>
       <c r="L31" s="2" t="inlineStr">
         <is>
-          <t>*</t>
+          <t>***</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>US only, Post-GenAI (&gt;=2023)</t>
+          <t>Post-GenAI (&gt;=2023)</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
@@ -2326,53 +2318,57 @@
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>[-5,+60]</t>
+          <t>[-1,+1]</t>
         </is>
       </c>
       <c r="D32" s="2" t="n">
-        <v>310</v>
+        <v>333</v>
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>3.300</t>
+          <t>-0.796***</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>1.523</t>
+          <t>-4.076</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>0.1277</t>
+          <t>0.0000</t>
         </is>
       </c>
       <c r="H32" s="2" t="inlineStr">
         <is>
-          <t>1.104</t>
+          <t>-2.162</t>
         </is>
       </c>
       <c r="I32" s="2" t="inlineStr">
         <is>
-          <t>0.2706</t>
+          <t>0.0313</t>
         </is>
       </c>
       <c r="J32" s="2" t="inlineStr">
         <is>
-          <t>-0.230</t>
+          <t>-2.454</t>
         </is>
       </c>
       <c r="K32" s="2" t="inlineStr">
         <is>
-          <t>0.8178</t>
-        </is>
-      </c>
-      <c r="L32" s="2" t="inlineStr"/>
+          <t>0.0141</t>
+        </is>
+      </c>
+      <c r="L32" s="2" t="inlineStr">
+        <is>
+          <t>***</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>US only, Post-GenAI (&gt;=2023)</t>
+          <t>Post-GenAI (&gt;=2023)</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
@@ -2386,41 +2382,41 @@
         </is>
       </c>
       <c r="D33" s="2" t="n">
-        <v>310</v>
+        <v>333</v>
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>-0.298**</t>
+          <t>-0.258**</t>
         </is>
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>-2.338</t>
+          <t>-2.102</t>
         </is>
       </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t>0.0194</t>
+          <t>0.0356</t>
         </is>
       </c>
       <c r="H33" s="2" t="inlineStr">
         <is>
-          <t>-1.622</t>
+          <t>-1.465</t>
         </is>
       </c>
       <c r="I33" s="2" t="inlineStr">
         <is>
-          <t>0.1059</t>
+          <t>0.1439</t>
         </is>
       </c>
       <c r="J33" s="2" t="inlineStr">
         <is>
-          <t>-2.461</t>
+          <t>-2.170</t>
         </is>
       </c>
       <c r="K33" s="2" t="inlineStr">
         <is>
-          <t>0.0139</t>
+          <t>0.0300</t>
         </is>
       </c>
       <c r="L33" s="2" t="inlineStr">
@@ -2432,7 +2428,7 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>US only, Post-GenAI (&gt;=2023)</t>
+          <t>Post-GenAI (&gt;=2023)</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
@@ -2442,57 +2438,53 @@
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>[0,+1]</t>
+          <t>[0,+20]</t>
         </is>
       </c>
       <c r="D34" s="2" t="n">
-        <v>310</v>
+        <v>333</v>
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>-0.661***</t>
+          <t>0.901</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>-4.251</t>
+          <t>0.354</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>0.0000</t>
+          <t>0.7232</t>
         </is>
       </c>
       <c r="H34" s="2" t="inlineStr">
         <is>
-          <t>-1.936</t>
+          <t>0.263</t>
         </is>
       </c>
       <c r="I34" s="2" t="inlineStr">
         <is>
-          <t>0.0538</t>
+          <t>0.7929</t>
         </is>
       </c>
       <c r="J34" s="2" t="inlineStr">
         <is>
-          <t>-2.396</t>
+          <t>-0.630</t>
         </is>
       </c>
       <c r="K34" s="2" t="inlineStr">
         <is>
-          <t>0.0166</t>
-        </is>
-      </c>
-      <c r="L34" s="2" t="inlineStr">
-        <is>
-          <t>***</t>
-        </is>
-      </c>
+          <t>0.5290</t>
+        </is>
+      </c>
+      <c r="L34" s="2" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>US only, Post-GenAI (&gt;=2023)</t>
+          <t>Post-GenAI (&gt;=2023)</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
@@ -2502,53 +2494,57 @@
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>[0,+20]</t>
+          <t>[0,+5]</t>
         </is>
       </c>
       <c r="D35" s="2" t="n">
-        <v>310</v>
+        <v>333</v>
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>0.873</t>
+          <t>-0.406**</t>
         </is>
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>0.083</t>
+          <t>-2.540</t>
         </is>
       </c>
       <c r="G35" s="2" t="inlineStr">
         <is>
-          <t>0.9340</t>
+          <t>0.0111</t>
         </is>
       </c>
       <c r="H35" s="2" t="inlineStr">
         <is>
-          <t>0.061</t>
+          <t>-1.594</t>
         </is>
       </c>
       <c r="I35" s="2" t="inlineStr">
         <is>
-          <t>0.9516</t>
+          <t>0.1119</t>
         </is>
       </c>
       <c r="J35" s="2" t="inlineStr">
         <is>
-          <t>-1.025</t>
+          <t>-1.863</t>
         </is>
       </c>
       <c r="K35" s="2" t="inlineStr">
         <is>
-          <t>0.3052</t>
-        </is>
-      </c>
-      <c r="L35" s="2" t="inlineStr"/>
+          <t>0.0624</t>
+        </is>
+      </c>
+      <c r="L35" s="2" t="inlineStr">
+        <is>
+          <t>**</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>US only, Post-GenAI (&gt;=2023)</t>
+          <t>Post-GenAI (&gt;=2023)</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
@@ -2558,57 +2554,57 @@
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>[0,+5]</t>
+          <t>[0,+60]</t>
         </is>
       </c>
       <c r="D36" s="2" t="n">
-        <v>310</v>
+        <v>333</v>
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>-0.475***</t>
+          <t>3.677**</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>-2.829</t>
+          <t>2.257</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t>0.0047</t>
+          <t>0.0240</t>
         </is>
       </c>
       <c r="H36" s="2" t="inlineStr">
         <is>
-          <t>-1.748</t>
+          <t>1.618</t>
         </is>
       </c>
       <c r="I36" s="2" t="inlineStr">
         <is>
-          <t>0.0814</t>
+          <t>0.1067</t>
         </is>
       </c>
       <c r="J36" s="2" t="inlineStr">
         <is>
-          <t>-2.160</t>
+          <t>0.776</t>
         </is>
       </c>
       <c r="K36" s="2" t="inlineStr">
         <is>
-          <t>0.0308</t>
+          <t>0.4377</t>
         </is>
       </c>
       <c r="L36" s="2" t="inlineStr">
         <is>
-          <t>***</t>
+          <t>**</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>US only, Pre-GenAI (&lt;=2022)</t>
+          <t>Pre-GenAI (&lt;=2022)</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
@@ -2622,53 +2618,53 @@
         </is>
       </c>
       <c r="D37" s="2" t="n">
-        <v>119</v>
+        <v>135</v>
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>-0.878**</t>
+          <t>-0.503*</t>
         </is>
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>-2.508</t>
+          <t>-1.885</t>
         </is>
       </c>
       <c r="G37" s="2" t="inlineStr">
         <is>
-          <t>0.0121</t>
+          <t>0.0595</t>
         </is>
       </c>
       <c r="H37" s="2" t="inlineStr">
         <is>
-          <t>-0.999</t>
+          <t>-0.775</t>
         </is>
       </c>
       <c r="I37" s="2" t="inlineStr">
         <is>
-          <t>0.3200</t>
+          <t>0.4400</t>
         </is>
       </c>
       <c r="J37" s="2" t="inlineStr">
         <is>
-          <t>-1.624</t>
+          <t>-0.965</t>
         </is>
       </c>
       <c r="K37" s="2" t="inlineStr">
         <is>
-          <t>0.1043</t>
+          <t>0.3348</t>
         </is>
       </c>
       <c r="L37" s="2" t="inlineStr">
         <is>
-          <t>**</t>
+          <t>*</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>US only, Pre-GenAI (&lt;=2022)</t>
+          <t>Pre-GenAI (&lt;=2022)</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
@@ -2678,57 +2674,53 @@
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>[-20,+60]</t>
+          <t>[0,+10]</t>
         </is>
       </c>
       <c r="D38" s="2" t="n">
-        <v>119</v>
+        <v>135</v>
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>7.718***</t>
+          <t>1.684</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>3.156</t>
+          <t>1.641</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
         <is>
-          <t>0.0016</t>
+          <t>0.1007</t>
         </is>
       </c>
       <c r="H38" s="2" t="inlineStr">
         <is>
-          <t>2.339</t>
+          <t>0.954</t>
         </is>
       </c>
       <c r="I38" s="2" t="inlineStr">
         <is>
-          <t>0.0210</t>
+          <t>0.3416</t>
         </is>
       </c>
       <c r="J38" s="2" t="inlineStr">
         <is>
-          <t>0.519</t>
+          <t>-0.042</t>
         </is>
       </c>
       <c r="K38" s="2" t="inlineStr">
         <is>
-          <t>0.6039</t>
-        </is>
-      </c>
-      <c r="L38" s="2" t="inlineStr">
-        <is>
-          <t>***</t>
-        </is>
-      </c>
+          <t>0.9666</t>
+        </is>
+      </c>
+      <c r="L38" s="2" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>US only, Pre-GenAI (&lt;=2022)</t>
+          <t>Pre-GenAI (&lt;=2022)</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
@@ -2738,45 +2730,45 @@
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>[-5,+60]</t>
+          <t>[0,+20]</t>
         </is>
       </c>
       <c r="D39" s="2" t="n">
-        <v>119</v>
+        <v>135</v>
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>9.779***</t>
+          <t>3.938***</t>
         </is>
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>4.426</t>
+          <t>2.890</t>
         </is>
       </c>
       <c r="G39" s="2" t="inlineStr">
         <is>
-          <t>0.0000</t>
+          <t>0.0038</t>
         </is>
       </c>
       <c r="H39" s="2" t="inlineStr">
         <is>
-          <t>2.967</t>
+          <t>1.873</t>
         </is>
       </c>
       <c r="I39" s="2" t="inlineStr">
         <is>
-          <t>0.0036</t>
+          <t>0.0632</t>
         </is>
       </c>
       <c r="J39" s="2" t="inlineStr">
         <is>
-          <t>0.886</t>
+          <t>0.701</t>
         </is>
       </c>
       <c r="K39" s="2" t="inlineStr">
         <is>
-          <t>0.3755</t>
+          <t>0.4831</t>
         </is>
       </c>
       <c r="L39" s="2" t="inlineStr">
@@ -2788,7 +2780,7 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>US only, Pre-GenAI (&lt;=2022)</t>
+          <t>Pre-GenAI (&lt;=2022)</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
@@ -2798,45 +2790,45 @@
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>[0,+10]</t>
+          <t>[0,+5]</t>
         </is>
       </c>
       <c r="D40" s="2" t="n">
-        <v>119</v>
+        <v>135</v>
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>1.113</t>
+          <t>-0.660</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>1.183</t>
+          <t>-1.065</t>
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr">
         <is>
-          <t>0.2369</t>
+          <t>0.2868</t>
         </is>
       </c>
       <c r="H40" s="2" t="inlineStr">
         <is>
-          <t>0.686</t>
+          <t>-0.606</t>
         </is>
       </c>
       <c r="I40" s="2" t="inlineStr">
         <is>
-          <t>0.4939</t>
+          <t>0.5453</t>
         </is>
       </c>
       <c r="J40" s="2" t="inlineStr">
         <is>
-          <t>-0.327</t>
+          <t>-1.252</t>
         </is>
       </c>
       <c r="K40" s="2" t="inlineStr">
         <is>
-          <t>0.7435</t>
+          <t>0.2107</t>
         </is>
       </c>
       <c r="L40" s="2" t="inlineStr"/>
@@ -2844,7 +2836,7 @@
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>US only, Pre-GenAI (&lt;=2022)</t>
+          <t>Pre-GenAI (&lt;=2022)</t>
         </is>
       </c>
       <c r="B41" s="2" t="inlineStr">
@@ -2854,45 +2846,45 @@
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>[0,+1]</t>
+          <t>[0,+60]</t>
         </is>
       </c>
       <c r="D41" s="2" t="n">
-        <v>119</v>
+        <v>135</v>
       </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t>-0.800***</t>
+          <t>10.862***</t>
         </is>
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>-2.605</t>
+          <t>5.051</t>
         </is>
       </c>
       <c r="G41" s="2" t="inlineStr">
         <is>
-          <t>0.0092</t>
+          <t>0.0000</t>
         </is>
       </c>
       <c r="H41" s="2" t="inlineStr">
         <is>
-          <t>-0.965</t>
+          <t>3.291</t>
         </is>
       </c>
       <c r="I41" s="2" t="inlineStr">
         <is>
-          <t>0.3363</t>
+          <t>0.0013</t>
         </is>
       </c>
       <c r="J41" s="2" t="inlineStr">
         <is>
-          <t>-1.337</t>
+          <t>1.221</t>
         </is>
       </c>
       <c r="K41" s="2" t="inlineStr">
         <is>
-          <t>0.1811</t>
+          <t>0.2220</t>
         </is>
       </c>
       <c r="L41" s="2" t="inlineStr">
@@ -2904,7 +2896,7 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>US only, Pre-GenAI (&lt;=2022)</t>
+          <t>Condition A (FF4)</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
@@ -2914,45 +2906,45 @@
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>[0,+20]</t>
+          <t>[-1,+1]</t>
         </is>
       </c>
       <c r="D42" s="2" t="n">
-        <v>119</v>
+        <v>263</v>
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>2.414**</t>
+          <t>-0.451**</t>
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>1.969</t>
+          <t>-2.392</t>
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr">
         <is>
-          <t>0.0490</t>
+          <t>0.0168</t>
         </is>
       </c>
       <c r="H42" s="2" t="inlineStr">
         <is>
-          <t>1.311</t>
+          <t>-1.084</t>
         </is>
       </c>
       <c r="I42" s="2" t="inlineStr">
         <is>
-          <t>0.1925</t>
+          <t>0.2795</t>
         </is>
       </c>
       <c r="J42" s="2" t="inlineStr">
         <is>
-          <t>-0.026</t>
+          <t>-1.937</t>
         </is>
       </c>
       <c r="K42" s="2" t="inlineStr">
         <is>
-          <t>0.9794</t>
+          <t>0.0528</t>
         </is>
       </c>
       <c r="L42" s="2" t="inlineStr">
@@ -2964,7 +2956,7 @@
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>US only, Pre-GenAI (&lt;=2022)</t>
+          <t>Condition A (FF4)</t>
         </is>
       </c>
       <c r="B43" s="2" t="inlineStr">
@@ -2974,57 +2966,57 @@
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>[0,+5]</t>
+          <t>[0,+10]</t>
         </is>
       </c>
       <c r="D43" s="2" t="n">
-        <v>119</v>
+        <v>263</v>
       </c>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t>-1.136*</t>
+          <t>0.148**</t>
         </is>
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>-1.636</t>
+          <t>-0.982</t>
         </is>
       </c>
       <c r="G43" s="2" t="inlineStr">
         <is>
-          <t>0.1018</t>
+          <t>0.3260</t>
         </is>
       </c>
       <c r="H43" s="2" t="inlineStr">
         <is>
-          <t>-0.921</t>
+          <t>-0.653</t>
         </is>
       </c>
       <c r="I43" s="2" t="inlineStr">
         <is>
-          <t>0.3589</t>
+          <t>0.5141</t>
         </is>
       </c>
       <c r="J43" s="2" t="inlineStr">
         <is>
-          <t>-1.697</t>
+          <t>-2.215</t>
         </is>
       </c>
       <c r="K43" s="2" t="inlineStr">
         <is>
-          <t>0.0896</t>
+          <t>0.0268</t>
         </is>
       </c>
       <c r="L43" s="2" t="inlineStr">
         <is>
-          <t>*</t>
+          <t>**</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>Post-GenAI (&gt;=2023)</t>
+          <t>Condition A (FF4)</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
@@ -3034,57 +3026,53 @@
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>[-1,+1]</t>
+          <t>[0,+20]</t>
         </is>
       </c>
       <c r="D44" s="2" t="n">
-        <v>333</v>
+        <v>263</v>
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>-0.796***</t>
+          <t>1.153</t>
         </is>
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>-4.076</t>
+          <t>0.737</t>
         </is>
       </c>
       <c r="G44" s="2" t="inlineStr">
         <is>
-          <t>0.0000</t>
+          <t>0.4613</t>
         </is>
       </c>
       <c r="H44" s="2" t="inlineStr">
         <is>
-          <t>-2.162</t>
+          <t>0.527</t>
         </is>
       </c>
       <c r="I44" s="2" t="inlineStr">
         <is>
-          <t>0.0313</t>
+          <t>0.5987</t>
         </is>
       </c>
       <c r="J44" s="2" t="inlineStr">
         <is>
-          <t>-2.453</t>
+          <t>-1.105</t>
         </is>
       </c>
       <c r="K44" s="2" t="inlineStr">
         <is>
-          <t>0.0142</t>
-        </is>
-      </c>
-      <c r="L44" s="2" t="inlineStr">
-        <is>
-          <t>***</t>
-        </is>
-      </c>
+          <t>0.2691</t>
+        </is>
+      </c>
+      <c r="L44" s="2" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>Post-GenAI (&gt;=2023)</t>
+          <t>Condition A (FF4)</t>
         </is>
       </c>
       <c r="B45" s="2" t="inlineStr">
@@ -3094,57 +3082,53 @@
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>[-20,+60]</t>
+          <t>[0,+5]</t>
         </is>
       </c>
       <c r="D45" s="2" t="n">
-        <v>333</v>
+        <v>263</v>
       </c>
       <c r="E45" s="2" t="inlineStr">
         <is>
-          <t>3.510*</t>
+          <t>0.305</t>
         </is>
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
-          <t>1.832</t>
+          <t>-0.782</t>
         </is>
       </c>
       <c r="G45" s="2" t="inlineStr">
         <is>
-          <t>0.0669</t>
+          <t>0.4340</t>
         </is>
       </c>
       <c r="H45" s="2" t="inlineStr">
         <is>
-          <t>1.345</t>
+          <t>-0.459</t>
         </is>
       </c>
       <c r="I45" s="2" t="inlineStr">
         <is>
-          <t>0.1796</t>
+          <t>0.6469</t>
         </is>
       </c>
       <c r="J45" s="2" t="inlineStr">
         <is>
-          <t>0.442</t>
+          <t>-1.165</t>
         </is>
       </c>
       <c r="K45" s="2" t="inlineStr">
         <is>
-          <t>0.6585</t>
-        </is>
-      </c>
-      <c r="L45" s="2" t="inlineStr">
-        <is>
-          <t>*</t>
-        </is>
-      </c>
+          <t>0.2441</t>
+        </is>
+      </c>
+      <c r="L45" s="2" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>Post-GenAI (&gt;=2023)</t>
+          <t>Condition A (FF4)</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
@@ -3154,700 +3138,52 @@
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>[-5,+60]</t>
+          <t>[0,+60]</t>
         </is>
       </c>
       <c r="D46" s="2" t="n">
-        <v>333</v>
+        <v>263</v>
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>3.286*</t>
+          <t>5.000***</t>
         </is>
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>1.717</t>
+          <t>3.202</t>
         </is>
       </c>
       <c r="G46" s="2" t="inlineStr">
         <is>
-          <t>0.0860</t>
+          <t>0.0014</t>
         </is>
       </c>
       <c r="H46" s="2" t="inlineStr">
         <is>
-          <t>1.249</t>
+          <t>2.427</t>
         </is>
       </c>
       <c r="I46" s="2" t="inlineStr">
         <is>
-          <t>0.2124</t>
+          <t>0.0159</t>
         </is>
       </c>
       <c r="J46" s="2" t="inlineStr">
         <is>
-          <t>0.149</t>
+          <t>1.277</t>
         </is>
       </c>
       <c r="K46" s="2" t="inlineStr">
         <is>
-          <t>0.8817</t>
+          <t>0.2014</t>
         </is>
       </c>
       <c r="L46" s="2" t="inlineStr">
         <is>
-          <t>*</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="2" t="inlineStr">
-        <is>
-          <t>Post-GenAI (&gt;=2023)</t>
-        </is>
-      </c>
-      <c r="B47" s="2" t="inlineStr">
-        <is>
-          <t>FF4</t>
-        </is>
-      </c>
-      <c r="C47" s="2" t="inlineStr">
-        <is>
-          <t>[0,+10]</t>
-        </is>
-      </c>
-      <c r="D47" s="2" t="n">
-        <v>333</v>
-      </c>
-      <c r="E47" s="2" t="inlineStr">
-        <is>
-          <t>-0.258**</t>
-        </is>
-      </c>
-      <c r="F47" s="2" t="inlineStr">
-        <is>
-          <t>-2.102</t>
-        </is>
-      </c>
-      <c r="G47" s="2" t="inlineStr">
-        <is>
-          <t>0.0356</t>
-        </is>
-      </c>
-      <c r="H47" s="2" t="inlineStr">
-        <is>
-          <t>-1.465</t>
-        </is>
-      </c>
-      <c r="I47" s="2" t="inlineStr">
-        <is>
-          <t>0.1439</t>
-        </is>
-      </c>
-      <c r="J47" s="2" t="inlineStr">
-        <is>
-          <t>-2.184</t>
-        </is>
-      </c>
-      <c r="K47" s="2" t="inlineStr">
-        <is>
-          <t>0.0290</t>
-        </is>
-      </c>
-      <c r="L47" s="2" t="inlineStr">
-        <is>
-          <t>**</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="2" t="inlineStr">
-        <is>
-          <t>Post-GenAI (&gt;=2023)</t>
-        </is>
-      </c>
-      <c r="B48" s="2" t="inlineStr">
-        <is>
-          <t>FF4</t>
-        </is>
-      </c>
-      <c r="C48" s="2" t="inlineStr">
-        <is>
-          <t>[0,+1]</t>
-        </is>
-      </c>
-      <c r="D48" s="2" t="n">
-        <v>333</v>
-      </c>
-      <c r="E48" s="2" t="inlineStr">
-        <is>
-          <t>-0.577***</t>
-        </is>
-      </c>
-      <c r="F48" s="2" t="inlineStr">
-        <is>
-          <t>-3.891</t>
-        </is>
-      </c>
-      <c r="G48" s="2" t="inlineStr">
-        <is>
-          <t>0.0001</t>
-        </is>
-      </c>
-      <c r="H48" s="2" t="inlineStr">
-        <is>
-          <t>-1.793</t>
-        </is>
-      </c>
-      <c r="I48" s="2" t="inlineStr">
-        <is>
-          <t>0.0738</t>
-        </is>
-      </c>
-      <c r="J48" s="2" t="inlineStr">
-        <is>
-          <t>-2.205</t>
-        </is>
-      </c>
-      <c r="K48" s="2" t="inlineStr">
-        <is>
-          <t>0.0275</t>
-        </is>
-      </c>
-      <c r="L48" s="2" t="inlineStr">
-        <is>
           <t>***</t>
         </is>
       </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="2" t="inlineStr">
-        <is>
-          <t>Post-GenAI (&gt;=2023)</t>
-        </is>
-      </c>
-      <c r="B49" s="2" t="inlineStr">
-        <is>
-          <t>FF4</t>
-        </is>
-      </c>
-      <c r="C49" s="2" t="inlineStr">
-        <is>
-          <t>[0,+20]</t>
-        </is>
-      </c>
-      <c r="D49" s="2" t="n">
-        <v>333</v>
-      </c>
-      <c r="E49" s="2" t="inlineStr">
-        <is>
-          <t>0.901</t>
-        </is>
-      </c>
-      <c r="F49" s="2" t="inlineStr">
-        <is>
-          <t>0.354</t>
-        </is>
-      </c>
-      <c r="G49" s="2" t="inlineStr">
-        <is>
-          <t>0.7232</t>
-        </is>
-      </c>
-      <c r="H49" s="2" t="inlineStr">
-        <is>
-          <t>0.263</t>
-        </is>
-      </c>
-      <c r="I49" s="2" t="inlineStr">
-        <is>
-          <t>0.7929</t>
-        </is>
-      </c>
-      <c r="J49" s="2" t="inlineStr">
-        <is>
-          <t>-0.649</t>
-        </is>
-      </c>
-      <c r="K49" s="2" t="inlineStr">
-        <is>
-          <t>0.5162</t>
-        </is>
-      </c>
-      <c r="L49" s="2" t="inlineStr"/>
-    </row>
-    <row r="50">
-      <c r="A50" s="2" t="inlineStr">
-        <is>
-          <t>Post-GenAI (&gt;=2023)</t>
-        </is>
-      </c>
-      <c r="B50" s="2" t="inlineStr">
-        <is>
-          <t>FF4</t>
-        </is>
-      </c>
-      <c r="C50" s="2" t="inlineStr">
-        <is>
-          <t>[0,+5]</t>
-        </is>
-      </c>
-      <c r="D50" s="2" t="n">
-        <v>333</v>
-      </c>
-      <c r="E50" s="2" t="inlineStr">
-        <is>
-          <t>-0.406**</t>
-        </is>
-      </c>
-      <c r="F50" s="2" t="inlineStr">
-        <is>
-          <t>-2.540</t>
-        </is>
-      </c>
-      <c r="G50" s="2" t="inlineStr">
-        <is>
-          <t>0.0111</t>
-        </is>
-      </c>
-      <c r="H50" s="2" t="inlineStr">
-        <is>
-          <t>-1.594</t>
-        </is>
-      </c>
-      <c r="I50" s="2" t="inlineStr">
-        <is>
-          <t>0.1119</t>
-        </is>
-      </c>
-      <c r="J50" s="2" t="inlineStr">
-        <is>
-          <t>-1.873</t>
-        </is>
-      </c>
-      <c r="K50" s="2" t="inlineStr">
-        <is>
-          <t>0.0611</t>
-        </is>
-      </c>
-      <c r="L50" s="2" t="inlineStr">
-        <is>
-          <t>**</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" s="2" t="inlineStr">
-        <is>
-          <t>Pre-GenAI (&lt;=2022)</t>
-        </is>
-      </c>
-      <c r="B51" s="2" t="inlineStr">
-        <is>
-          <t>FF4</t>
-        </is>
-      </c>
-      <c r="C51" s="2" t="inlineStr">
-        <is>
-          <t>[-1,+1]</t>
-        </is>
-      </c>
-      <c r="D51" s="2" t="n">
-        <v>134</v>
-      </c>
-      <c r="E51" s="2" t="inlineStr">
-        <is>
-          <t>-0.481*</t>
-        </is>
-      </c>
-      <c r="F51" s="2" t="inlineStr">
-        <is>
-          <t>-1.843</t>
-        </is>
-      </c>
-      <c r="G51" s="2" t="inlineStr">
-        <is>
-          <t>0.0653</t>
-        </is>
-      </c>
-      <c r="H51" s="2" t="inlineStr">
-        <is>
-          <t>-0.755</t>
-        </is>
-      </c>
-      <c r="I51" s="2" t="inlineStr">
-        <is>
-          <t>0.4518</t>
-        </is>
-      </c>
-      <c r="J51" s="2" t="inlineStr">
-        <is>
-          <t>-0.956</t>
-        </is>
-      </c>
-      <c r="K51" s="2" t="inlineStr">
-        <is>
-          <t>0.3392</t>
-        </is>
-      </c>
-      <c r="L51" s="2" t="inlineStr">
-        <is>
-          <t>*</t>
-        </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" s="2" t="inlineStr">
-        <is>
-          <t>Pre-GenAI (&lt;=2022)</t>
-        </is>
-      </c>
-      <c r="B52" s="2" t="inlineStr">
-        <is>
-          <t>FF4</t>
-        </is>
-      </c>
-      <c r="C52" s="2" t="inlineStr">
-        <is>
-          <t>[-20,+60]</t>
-        </is>
-      </c>
-      <c r="D52" s="2" t="n">
-        <v>134</v>
-      </c>
-      <c r="E52" s="2" t="inlineStr">
-        <is>
-          <t>9.673***</t>
-        </is>
-      </c>
-      <c r="F52" s="2" t="inlineStr">
-        <is>
-          <t>3.798</t>
-        </is>
-      </c>
-      <c r="G52" s="2" t="inlineStr">
-        <is>
-          <t>0.0001</t>
-        </is>
-      </c>
-      <c r="H52" s="2" t="inlineStr">
-        <is>
-          <t>2.678</t>
-        </is>
-      </c>
-      <c r="I52" s="2" t="inlineStr">
-        <is>
-          <t>0.0083</t>
-        </is>
-      </c>
-      <c r="J52" s="2" t="inlineStr">
-        <is>
-          <t>0.929</t>
-        </is>
-      </c>
-      <c r="K52" s="2" t="inlineStr">
-        <is>
-          <t>0.3531</t>
-        </is>
-      </c>
-      <c r="L52" s="2" t="inlineStr">
-        <is>
-          <t>***</t>
-        </is>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" s="2" t="inlineStr">
-        <is>
-          <t>Pre-GenAI (&lt;=2022)</t>
-        </is>
-      </c>
-      <c r="B53" s="2" t="inlineStr">
-        <is>
-          <t>FF4</t>
-        </is>
-      </c>
-      <c r="C53" s="2" t="inlineStr">
-        <is>
-          <t>[-5,+60]</t>
-        </is>
-      </c>
-      <c r="D53" s="2" t="n">
-        <v>134</v>
-      </c>
-      <c r="E53" s="2" t="inlineStr">
-        <is>
-          <t>11.487***</t>
-        </is>
-      </c>
-      <c r="F53" s="2" t="inlineStr">
-        <is>
-          <t>5.062</t>
-        </is>
-      </c>
-      <c r="G53" s="2" t="inlineStr">
-        <is>
-          <t>0.0000</t>
-        </is>
-      </c>
-      <c r="H53" s="2" t="inlineStr">
-        <is>
-          <t>3.294</t>
-        </is>
-      </c>
-      <c r="I53" s="2" t="inlineStr">
-        <is>
-          <t>0.0013</t>
-        </is>
-      </c>
-      <c r="J53" s="2" t="inlineStr">
-        <is>
-          <t>1.224</t>
-        </is>
-      </c>
-      <c r="K53" s="2" t="inlineStr">
-        <is>
-          <t>0.2209</t>
-        </is>
-      </c>
-      <c r="L53" s="2" t="inlineStr">
-        <is>
-          <t>***</t>
-        </is>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" s="2" t="inlineStr">
-        <is>
-          <t>Pre-GenAI (&lt;=2022)</t>
-        </is>
-      </c>
-      <c r="B54" s="2" t="inlineStr">
-        <is>
-          <t>FF4</t>
-        </is>
-      </c>
-      <c r="C54" s="2" t="inlineStr">
-        <is>
-          <t>[0,+10]</t>
-        </is>
-      </c>
-      <c r="D54" s="2" t="n">
-        <v>134</v>
-      </c>
-      <c r="E54" s="2" t="inlineStr">
-        <is>
-          <t>1.673</t>
-        </is>
-      </c>
-      <c r="F54" s="2" t="inlineStr">
-        <is>
-          <t>1.622</t>
-        </is>
-      </c>
-      <c r="G54" s="2" t="inlineStr">
-        <is>
-          <t>0.1047</t>
-        </is>
-      </c>
-      <c r="H54" s="2" t="inlineStr">
-        <is>
-          <t>0.940</t>
-        </is>
-      </c>
-      <c r="I54" s="2" t="inlineStr">
-        <is>
-          <t>0.3490</t>
-        </is>
-      </c>
-      <c r="J54" s="2" t="inlineStr">
-        <is>
-          <t>-0.126</t>
-        </is>
-      </c>
-      <c r="K54" s="2" t="inlineStr">
-        <is>
-          <t>0.8994</t>
-        </is>
-      </c>
-      <c r="L54" s="2" t="inlineStr"/>
-    </row>
-    <row r="55">
-      <c r="A55" s="2" t="inlineStr">
-        <is>
-          <t>Pre-GenAI (&lt;=2022)</t>
-        </is>
-      </c>
-      <c r="B55" s="2" t="inlineStr">
-        <is>
-          <t>FF4</t>
-        </is>
-      </c>
-      <c r="C55" s="2" t="inlineStr">
-        <is>
-          <t>[0,+1]</t>
-        </is>
-      </c>
-      <c r="D55" s="2" t="n">
-        <v>134</v>
-      </c>
-      <c r="E55" s="2" t="inlineStr">
-        <is>
-          <t>-0.489**</t>
-        </is>
-      </c>
-      <c r="F55" s="2" t="inlineStr">
-        <is>
-          <t>-1.974</t>
-        </is>
-      </c>
-      <c r="G55" s="2" t="inlineStr">
-        <is>
-          <t>0.0484</t>
-        </is>
-      </c>
-      <c r="H55" s="2" t="inlineStr">
-        <is>
-          <t>-0.751</t>
-        </is>
-      </c>
-      <c r="I55" s="2" t="inlineStr">
-        <is>
-          <t>0.4538</t>
-        </is>
-      </c>
-      <c r="J55" s="2" t="inlineStr">
-        <is>
-          <t>-0.761</t>
-        </is>
-      </c>
-      <c r="K55" s="2" t="inlineStr">
-        <is>
-          <t>0.4468</t>
-        </is>
-      </c>
-      <c r="L55" s="2" t="inlineStr">
-        <is>
-          <t>**</t>
-        </is>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" s="2" t="inlineStr">
-        <is>
-          <t>Pre-GenAI (&lt;=2022)</t>
-        </is>
-      </c>
-      <c r="B56" s="2" t="inlineStr">
-        <is>
-          <t>FF4</t>
-        </is>
-      </c>
-      <c r="C56" s="2" t="inlineStr">
-        <is>
-          <t>[0,+20]</t>
-        </is>
-      </c>
-      <c r="D56" s="2" t="n">
-        <v>134</v>
-      </c>
-      <c r="E56" s="2" t="inlineStr">
-        <is>
-          <t>3.898***</t>
-        </is>
-      </c>
-      <c r="F56" s="2" t="inlineStr">
-        <is>
-          <t>2.849</t>
-        </is>
-      </c>
-      <c r="G56" s="2" t="inlineStr">
-        <is>
-          <t>0.0044</t>
-        </is>
-      </c>
-      <c r="H56" s="2" t="inlineStr">
-        <is>
-          <t>1.840</t>
-        </is>
-      </c>
-      <c r="I56" s="2" t="inlineStr">
-        <is>
-          <t>0.0680</t>
-        </is>
-      </c>
-      <c r="J56" s="2" t="inlineStr">
-        <is>
-          <t>0.590</t>
-        </is>
-      </c>
-      <c r="K56" s="2" t="inlineStr">
-        <is>
-          <t>0.5552</t>
-        </is>
-      </c>
-      <c r="L56" s="2" t="inlineStr">
-        <is>
-          <t>***</t>
-        </is>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" s="2" t="inlineStr">
-        <is>
-          <t>Pre-GenAI (&lt;=2022)</t>
-        </is>
-      </c>
-      <c r="B57" s="2" t="inlineStr">
-        <is>
-          <t>FF4</t>
-        </is>
-      </c>
-      <c r="C57" s="2" t="inlineStr">
-        <is>
-          <t>[0,+5]</t>
-        </is>
-      </c>
-      <c r="D57" s="2" t="n">
-        <v>134</v>
-      </c>
-      <c r="E57" s="2" t="inlineStr">
-        <is>
-          <t>-0.623</t>
-        </is>
-      </c>
-      <c r="F57" s="2" t="inlineStr">
-        <is>
-          <t>-1.012</t>
-        </is>
-      </c>
-      <c r="G57" s="2" t="inlineStr">
-        <is>
-          <t>0.3117</t>
-        </is>
-      </c>
-      <c r="H57" s="2" t="inlineStr">
-        <is>
-          <t>-0.574</t>
-        </is>
-      </c>
-      <c r="I57" s="2" t="inlineStr">
-        <is>
-          <t>0.5670</t>
-        </is>
-      </c>
-      <c r="J57" s="2" t="inlineStr">
-        <is>
-          <t>-1.223</t>
-        </is>
-      </c>
-      <c r="K57" s="2" t="inlineStr">
-        <is>
-          <t>0.2212</t>
-        </is>
-      </c>
-      <c r="L57" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -4088,7 +3424,7 @@
   <dimension ref="A1:M19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="13" customWidth="1" min="1" max="1"/>
     <col width="20" customWidth="1" min="2" max="2"/>
     <col width="21" customWidth="1" min="3" max="3"/>
     <col width="20" customWidth="1" min="4" max="4"/>
@@ -4188,42 +3524,42 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>3.845</t>
+          <t>8.655</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>(3.136)</t>
+          <t>(9.415)</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>0.881</t>
+          <t>0.040</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>(2.276)</t>
+          <t>(1.725)</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>-2.797</t>
+          <t>-9.629</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>(3.375)</t>
+          <t>(9.595)</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>-2.495</t>
+          <t>-1.028</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>(2.089)</t>
+          <t>(1.590)</t>
         </is>
       </c>
       <c r="L2" s="2" t="n">
@@ -4231,7 +3567,7 @@
       </c>
       <c r="M2" s="2" t="inlineStr">
         <is>
-          <t>0.017</t>
+          <t>0.014</t>
         </is>
       </c>
     </row>
@@ -4253,50 +3589,50 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>3.070</t>
+          <t>4.816</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>(2.011)</t>
+          <t>(4.026)</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>0.957</t>
+          <t>-0.088</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>(1.447)</t>
+          <t>(1.133)</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>-2.653</t>
+          <t>-5.265</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>(2.222)</t>
+          <t>(4.306)</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>-2.018</t>
+          <t>-0.720</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>(1.249)</t>
+          <t>(1.020)</t>
         </is>
       </c>
       <c r="L3" s="2" t="n">
-        <v>444</v>
+        <v>445</v>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>0.008</t>
+          <t>0.003</t>
         </is>
       </c>
     </row>
@@ -4318,42 +3654,42 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>3.327</t>
+          <t>6.691</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>(2.116)</t>
+          <t>(5.458)</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>1.592</t>
+          <t>0.413</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>(1.485)</t>
+          <t>(1.186)</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>-2.922</t>
+          <t>-7.119</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>(2.326)</t>
+          <t>(5.669)</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>-2.667**</t>
+          <t>-1.242</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
         <is>
-          <t>(1.285)</t>
+          <t>(1.073)</t>
         </is>
       </c>
       <c r="L4" s="2" t="n">
@@ -4361,7 +3697,7 @@
       </c>
       <c r="M4" s="2" t="inlineStr">
         <is>
-          <t>0.009</t>
+          <t>0.004</t>
         </is>
       </c>
     </row>
@@ -4383,50 +3719,50 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>4.607</t>
+          <t>-1.087</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>(4.744)</t>
+          <t>(4.232)</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>1.277</t>
+          <t>-0.689</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>(3.424)</t>
+          <t>(2.972)</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>-3.315</t>
+          <t>-1.512</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>(5.085)</t>
+          <t>(6.925)</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>-6.172</t>
+          <t>-4.677</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
         <is>
-          <t>(6.574)</t>
+          <t>(6.808)</t>
         </is>
       </c>
       <c r="L5" s="2" t="n">
-        <v>105</v>
+        <v>80</v>
       </c>
       <c r="M5" s="2" t="inlineStr">
         <is>
-          <t>0.050</t>
+          <t>0.082</t>
         </is>
       </c>
     </row>
@@ -4448,50 +3784,50 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>4.974*</t>
+          <t>2.006</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>(2.899)</t>
+          <t>(2.058)</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>3.267</t>
+          <t>1.939</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>(2.284)</t>
+          <t>(2.106)</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>-5.006</t>
+          <t>-2.714</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>(3.280)</t>
+          <t>(3.864)</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>-4.920</t>
+          <t>-4.656</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
         <is>
-          <t>(4.027)</t>
+          <t>(4.324)</t>
         </is>
       </c>
       <c r="L6" s="2" t="n">
-        <v>235</v>
+        <v>191</v>
       </c>
       <c r="M6" s="2" t="inlineStr">
         <is>
-          <t>0.023</t>
+          <t>0.038</t>
         </is>
       </c>
     </row>
@@ -4513,57 +3849,57 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>4.843*</t>
+          <t>2.006</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>(2.920)</t>
+          <t>(2.058)</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>3.328</t>
+          <t>1.939</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>(2.285)</t>
+          <t>(2.106)</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>-4.929</t>
+          <t>-2.714</t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>(3.288)</t>
+          <t>(3.864)</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>-4.921</t>
+          <t>-4.656</t>
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr">
         <is>
-          <t>(4.024)</t>
+          <t>(4.324)</t>
         </is>
       </c>
       <c r="L7" s="2" t="n">
-        <v>233</v>
+        <v>190</v>
       </c>
       <c r="M7" s="2" t="inlineStr">
         <is>
-          <t>0.023</t>
+          <t>0.036</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>CAR[-5,+30]</t>
+          <t>CAR[0,+20]</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
@@ -4578,42 +3914,42 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>-2.136</t>
+          <t>3.539</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>(9.852)</t>
+          <t>(37.572)</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>-5.415</t>
+          <t>-2.272</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>(6.873)</t>
+          <t>(4.152)</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>-4.226</t>
+          <t>3.339</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>(10.396)</t>
+          <t>(38.112)</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>10.778*</t>
+          <t>3.301</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr">
         <is>
-          <t>(6.465)</t>
+          <t>(3.961)</t>
         </is>
       </c>
       <c r="L8" s="2" t="n">
@@ -4621,14 +3957,14 @@
       </c>
       <c r="M8" s="2" t="inlineStr">
         <is>
-          <t>0.036</t>
+          <t>0.014</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>CAR[-5,+30]</t>
+          <t>CAR[0,+20]</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
@@ -4643,57 +3979,57 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>0.655</t>
+          <t>10.457</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>(5.059)</t>
+          <t>(20.843)</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>-3.008</t>
+          <t>-2.061</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>(3.649)</t>
+          <t>(2.188)</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>-4.315</t>
+          <t>-9.422</t>
         </is>
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>(5.530)</t>
+          <t>(21.359)</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>5.816*</t>
+          <t>2.843</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr">
         <is>
-          <t>(3.285)</t>
+          <t>(2.001)</t>
         </is>
       </c>
       <c r="L9" s="2" t="n">
-        <v>444</v>
+        <v>445</v>
       </c>
       <c r="M9" s="2" t="inlineStr">
         <is>
-          <t>0.016</t>
+          <t>0.007</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>CAR[-5,+30]</t>
+          <t>CAR[0,+20]</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
@@ -4708,42 +4044,42 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>1.809</t>
+          <t>20.941</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>(5.096)</t>
+          <t>(26.829)</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>-1.329</t>
+          <t>-0.701</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>(3.727)</t>
+          <t>(2.194)</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>-5.433</t>
+          <t>-19.960</t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>(5.581)</t>
+          <t>(27.232)</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>4.117</t>
+          <t>1.536</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr">
         <is>
-          <t>(3.359)</t>
+          <t>(2.000)</t>
         </is>
       </c>
       <c r="L10" s="2" t="n">
@@ -4751,14 +4087,14 @@
       </c>
       <c r="M10" s="2" t="inlineStr">
         <is>
-          <t>0.012</t>
+          <t>0.011</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>CAR[-5,+30]</t>
+          <t>CAR[0,+20]</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
@@ -4773,57 +4109,57 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>-1.631</t>
+          <t>-18.797</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>(13.298)</t>
+          <t>(16.164)</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>-4.901</t>
+          <t>-0.788</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>(9.452)</t>
+          <t>(7.339)</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>-5.472</t>
+          <t>35.453</t>
         </is>
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>(13.983)</t>
+          <t>(26.774)</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>7.468</t>
+          <t>-0.325</t>
         </is>
       </c>
       <c r="K11" s="2" t="inlineStr">
         <is>
-          <t>(12.643)</t>
+          <t>(15.153)</t>
         </is>
       </c>
       <c r="L11" s="2" t="n">
-        <v>105</v>
+        <v>80</v>
       </c>
       <c r="M11" s="2" t="inlineStr">
         <is>
-          <t>0.046</t>
+          <t>0.086</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>CAR[-5,+30]</t>
+          <t>CAR[0,+20]</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
@@ -4838,57 +4174,57 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>3.301</t>
+          <t>16.515</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>(6.351)</t>
+          <t>(50.744)</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>1.508</t>
+          <t>6.368*</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>(5.209)</t>
+          <t>(3.689)</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>-7.814</t>
+          <t>-19.496</t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>(7.119)</t>
+          <t>(52.791)</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>-5.992</t>
+          <t>-12.473</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr">
         <is>
-          <t>(8.408)</t>
+          <t>(8.770)</t>
         </is>
       </c>
       <c r="L12" s="2" t="n">
-        <v>235</v>
+        <v>191</v>
       </c>
       <c r="M12" s="2" t="inlineStr">
         <is>
-          <t>0.033</t>
+          <t>0.056</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>CAR[-5,+30]</t>
+          <t>CAR[0,+20]</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
@@ -4903,57 +4239,57 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>3.119</t>
+          <t>16.515</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>(6.388)</t>
+          <t>(50.744)</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>1.593</t>
+          <t>6.368*</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>(5.218)</t>
+          <t>(3.689)</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>-7.705</t>
+          <t>-19.496</t>
         </is>
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>(7.133)</t>
+          <t>(52.791)</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>-5.994</t>
+          <t>-12.473</t>
         </is>
       </c>
       <c r="K13" s="2" t="inlineStr">
         <is>
-          <t>(8.407)</t>
+          <t>(8.770)</t>
         </is>
       </c>
       <c r="L13" s="2" t="n">
-        <v>233</v>
+        <v>190</v>
       </c>
       <c r="M13" s="2" t="inlineStr">
         <is>
-          <t>0.033</t>
+          <t>0.056</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>CAR[0,+20]</t>
+          <t>CAR[0,+60]</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
@@ -4968,42 +4304,42 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>-7.195</t>
+          <t>-13.288</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>(7.886)</t>
+          <t>(28.063)</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>-3.820</t>
+          <t>-9.610*</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>(6.107)</t>
+          <t>(5.253)</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>4.156</t>
+          <t>20.156</t>
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>(8.296)</t>
+          <t>(29.142)</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>7.086</t>
+          <t>11.182**</t>
         </is>
       </c>
       <c r="K14" s="2" t="inlineStr">
         <is>
-          <t>(5.813)</t>
+          <t>(5.008)</t>
         </is>
       </c>
       <c r="L14" s="2" t="n">
@@ -5011,14 +4347,14 @@
       </c>
       <c r="M14" s="2" t="inlineStr">
         <is>
-          <t>0.017</t>
+          <t>0.034</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>CAR[0,+20]</t>
+          <t>CAR[0,+60]</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
@@ -5033,57 +4369,57 @@
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>-3.807</t>
+          <t>-17.513</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>(4.111)</t>
+          <t>(11.729)</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>-3.270</t>
+          <t>-4.839*</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>(2.874)</t>
+          <t>(2.635)</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>2.064</t>
+          <t>20.162</t>
         </is>
       </c>
       <c r="I15" s="2" t="inlineStr">
         <is>
-          <t>(4.478)</t>
+          <t>(12.831)</t>
         </is>
       </c>
       <c r="J15" s="2" t="inlineStr">
         <is>
-          <t>5.044**</t>
+          <t>6.005**</t>
         </is>
       </c>
       <c r="K15" s="2" t="inlineStr">
         <is>
-          <t>(2.573)</t>
+          <t>(2.409)</t>
         </is>
       </c>
       <c r="L15" s="2" t="n">
-        <v>444</v>
+        <v>445</v>
       </c>
       <c r="M15" s="2" t="inlineStr">
         <is>
-          <t>0.008</t>
+          <t>0.014</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>CAR[0,+20]</t>
+          <t>CAR[0,+60]</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
@@ -5098,42 +4434,42 @@
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>-2.823</t>
+          <t>-11.294</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>(4.129)</t>
+          <t>(14.974)</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>-1.715</t>
+          <t>-3.743</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>(2.920)</t>
+          <t>(2.659)</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>1.138</t>
+          <t>13.962</t>
         </is>
       </c>
       <c r="I16" s="2" t="inlineStr">
         <is>
-          <t>(4.508)</t>
+          <t>(15.853)</t>
         </is>
       </c>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>3.506</t>
+          <t>4.890**</t>
         </is>
       </c>
       <c r="K16" s="2" t="inlineStr">
         <is>
-          <t>(2.612)</t>
+          <t>(2.426)</t>
         </is>
       </c>
       <c r="L16" s="2" t="n">
@@ -5141,14 +4477,14 @@
       </c>
       <c r="M16" s="2" t="inlineStr">
         <is>
-          <t>0.004</t>
+          <t>0.007</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>CAR[0,+20]</t>
+          <t>CAR[0,+60]</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
@@ -5163,57 +4499,57 @@
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>-1.555</t>
+          <t>-26.024</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>(11.640)</t>
+          <t>(21.026)</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>0.924</t>
+          <t>-6.419</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>(8.768)</t>
+          <t>(8.643)</t>
         </is>
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>-3.244</t>
+          <t>44.851</t>
         </is>
       </c>
       <c r="I17" s="2" t="inlineStr">
         <is>
-          <t>(12.149)</t>
+          <t>(33.317)</t>
         </is>
       </c>
       <c r="J17" s="2" t="inlineStr">
         <is>
-          <t>0.284</t>
+          <t>5.782</t>
         </is>
       </c>
       <c r="K17" s="2" t="inlineStr">
         <is>
-          <t>(10.856)</t>
+          <t>(18.268)</t>
         </is>
       </c>
       <c r="L17" s="2" t="n">
-        <v>105</v>
+        <v>80</v>
       </c>
       <c r="M17" s="2" t="inlineStr">
         <is>
-          <t>0.018</t>
+          <t>0.100</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>CAR[0,+20]</t>
+          <t>CAR[0,+60]</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
@@ -5228,57 +4564,57 @@
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>0.154</t>
+          <t>-22.371***</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>(5.263)</t>
+          <t>(3.662)</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>1.678</t>
+          <t>3.486</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>(4.102)</t>
+          <t>(4.095)</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>-1.747</t>
+          <t>27.876*</t>
         </is>
       </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
-          <t>(5.799)</t>
+          <t>(14.753)</t>
         </is>
       </c>
       <c r="J18" s="2" t="inlineStr">
         <is>
-          <t>-5.169</t>
+          <t>-13.659</t>
         </is>
       </c>
       <c r="K18" s="2" t="inlineStr">
         <is>
-          <t>(7.474)</t>
+          <t>(9.492)</t>
         </is>
       </c>
       <c r="L18" s="2" t="n">
-        <v>235</v>
+        <v>191</v>
       </c>
       <c r="M18" s="2" t="inlineStr">
         <is>
-          <t>0.027</t>
+          <t>0.073</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>CAR[0,+20]</t>
+          <t>CAR[0,+60]</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
@@ -5293,50 +4629,50 @@
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>0.017</t>
+          <t>-22.371***</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>(5.296)</t>
+          <t>(3.662)</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>1.741</t>
+          <t>3.486</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>(4.111)</t>
+          <t>(4.095)</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>-1.666</t>
+          <t>27.876*</t>
         </is>
       </c>
       <c r="I19" s="2" t="inlineStr">
         <is>
-          <t>(5.810)</t>
+          <t>(14.753)</t>
         </is>
       </c>
       <c r="J19" s="2" t="inlineStr">
         <is>
-          <t>-5.170</t>
+          <t>-13.659</t>
         </is>
       </c>
       <c r="K19" s="2" t="inlineStr">
         <is>
-          <t>(7.474)</t>
+          <t>(9.492)</t>
         </is>
       </c>
       <c r="L19" s="2" t="n">
-        <v>233</v>
+        <v>190</v>
       </c>
       <c r="M19" s="2" t="inlineStr">
         <is>
-          <t>0.027</t>
+          <t>0.073</t>
         </is>
       </c>
     </row>

</xml_diff>